<commit_message>
fix: accept YouTube replay percentages
</commit_message>
<xml_diff>
--- a/docs/Social_MKT_Data_Hub_Multi_Channel_Blueprint_v0.10.2.xlsx
+++ b/docs/Social_MKT_Data_Hub_Multi_Channel_Blueprint_v0.10.2.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R99da5e1cc66e40ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Inventory" sheetId="2" r:id="Ref217fa88f164c90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Fields" sheetId="3" r:id="R7fb619e6f39f43f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ads Fields" sheetId="4" r:id="R5d23761d06d6477f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Select Options" sheetId="5" r:id="Rcd0b7883cfca48b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys &amp; Metrics" sheetId="6" r:id="R57a8ba522bd4475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT Checklist" sheetId="7" r:id="R77be464b29464764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R3199983b6b004105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Mapping" sheetId="9" r:id="Rb68998221d2841ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Approval" sheetId="10" r:id="R7cb214bc24eb4b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R95dbc04fb7504ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Inventory" sheetId="2" r:id="R410cea81afcd4f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Fields" sheetId="3" r:id="Raf3da51b928c4203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ads Fields" sheetId="4" r:id="R96c3758327914cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Select Options" sheetId="5" r:id="R635aad3aedf04cab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys &amp; Metrics" sheetId="6" r:id="R52e0e780c1894f13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT Checklist" sheetId="7" r:id="R070ef996935f4387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rdefc65bc0b7949fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Mapping" sheetId="9" r:id="Redb33e12afd44d51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Approval" sheetId="10" r:id="R9c4b196d11d94547"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1289,9 +1289,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2110,7 +2110,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f7e076e7cb945e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15e30e7e02b74821"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2510,7 +2510,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cdc55406984ca2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd921dc810bf94fa4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4012,7 +4012,7 @@
         <x:v>Analytics averageViewPercentage</x:v>
       </x:c>
       <x:c r="I45" s="101" t="str">
-        <x:v>Percentage value 0–100</x:v>
+        <x:v>Non-negative percentage; may exceed 100 when viewers rewatch portions</x:v>
       </x:c>
       <x:c r="J45" s="101" t="n">
         <x:v>52.4</x:v>
@@ -4098,7 +4098,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fa1649b7fa9474c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R657944a384d7485e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6359,7 +6359,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b86318adbd74e23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc58a9876b813414e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6935,7 +6935,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93ab35b0347a4594"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d5795a607634c13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7439,7 +7439,7 @@
         <x:v>Null when Source null</x:v>
       </x:c>
       <x:c r="F24" s="230" t="str">
-        <x:v>RAW retains percentage 0–100</x:v>
+        <x:v>RAW retains non-negative Source percentage; value may exceed 100</x:v>
       </x:c>
       <x:c r="G24" s="231" t="str">
         <x:v>52.4 ÷ 100 = 0.524</x:v>
@@ -7666,7 +7666,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4edb311c60c046a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58ad58b3b51d4b16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8246,7 +8246,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31e8131d952c42cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3989f69e169942b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8522,7 +8522,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4996d20526246e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf9ce09d39f9410c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9807,7 +9807,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re45d0e6388c64e7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43be70b1b347406e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: preserve YouTube signed daily counts
</commit_message>
<xml_diff>
--- a/docs/Social_MKT_Data_Hub_Multi_Channel_Blueprint_v0.10.2.xlsx
+++ b/docs/Social_MKT_Data_Hub_Multi_Channel_Blueprint_v0.10.2.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R95dbc04fb7504ebf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Inventory" sheetId="2" r:id="R410cea81afcd4f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Fields" sheetId="3" r:id="Raf3da51b928c4203"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ads Fields" sheetId="4" r:id="R96c3758327914cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Select Options" sheetId="5" r:id="R635aad3aedf04cab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys &amp; Metrics" sheetId="6" r:id="R52e0e780c1894f13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT Checklist" sheetId="7" r:id="R070ef996935f4387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="Rdefc65bc0b7949fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Mapping" sheetId="9" r:id="Redb33e12afd44d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Approval" sheetId="10" r:id="R9c4b196d11d94547"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R50ae1cecea514f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table Inventory" sheetId="2" r:id="Raa211d6071434770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Fields" sheetId="3" r:id="R9e31f23991d54757"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ads Fields" sheetId="4" r:id="R0a656cd0de8d46a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Select Options" sheetId="5" r:id="R666cfc919f7a4359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keys &amp; Metrics" sheetId="6" r:id="Rdac9efa20b644a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UAT Checklist" sheetId="7" r:id="R6e0fa61cefd64f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R498fedf11a4748aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Mapping" sheetId="9" r:id="R646d6421affa4374"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YouTube Approval" sheetId="10" r:id="Rd6ef7260e16a41a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2026,7 +2026,7 @@
         <x:v>Conversion contract incomplete</x:v>
       </x:c>
       <x:c r="C17" s="230" t="str">
-        <x:v>minutes×60; seconds direct; percentage÷100 only in future canonical layer</x:v>
+        <x:v>Signed daily counts preserved; minutes×60; seconds direct; percentage÷100 only in future canonical layer</x:v>
       </x:c>
       <x:c r="D17" s="236" t="str">
         <x:v>Technical Approved</x:v>
@@ -2110,7 +2110,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15e30e7e02b74821"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf6765a3184e49f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2510,7 +2510,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd921dc810bf94fa4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51f54cfd8e574eb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3802,13 +3802,13 @@
         <x:v>Analytics metric views</x:v>
       </x:c>
       <x:c r="I39" s="101" t="str">
-        <x:v>Views during Source day</x:v>
+        <x:v>Signed integer views during Source day</x:v>
       </x:c>
       <x:c r="J39" s="101" t="n">
         <x:v>120</x:v>
       </x:c>
       <x:c r="K39" s="101" t="str">
-        <x:v>Not cumulative</x:v>
+        <x:v>Preserve Provider adjustments; not cumulative</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="25.5" customHeight="1">
@@ -3837,13 +3837,13 @@
         <x:v>Analytics metric likes</x:v>
       </x:c>
       <x:c r="I40" s="97" t="str">
-        <x:v>Likes during Source day</x:v>
+        <x:v>Signed integer likes during Source day</x:v>
       </x:c>
       <x:c r="J40" s="97" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="K40" s="97" t="str">
-        <x:v>Missing stays null</x:v>
+        <x:v>Preserve Provider adjustments; missing stays null</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="25.5" customHeight="1">
@@ -3872,13 +3872,13 @@
         <x:v>Analytics metric comments</x:v>
       </x:c>
       <x:c r="I41" s="101" t="str">
-        <x:v>Comments during Source day</x:v>
+        <x:v>Signed integer comments during Source day</x:v>
       </x:c>
       <x:c r="J41" s="101" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="K41" s="101" t="str">
-        <x:v>Missing stays null</x:v>
+        <x:v>Preserve Provider adjustments; missing stays null</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="25.5" customHeight="1">
@@ -3907,13 +3907,13 @@
         <x:v>Analytics metric shares</x:v>
       </x:c>
       <x:c r="I42" s="97" t="str">
-        <x:v>Shares during Source day</x:v>
+        <x:v>Signed integer shares during Source day</x:v>
       </x:c>
       <x:c r="J42" s="97" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K42" s="97" t="str">
-        <x:v>Missing stays null</x:v>
+        <x:v>Preserve Provider adjustments; missing stays null</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="25.5" customHeight="1">
@@ -4098,7 +4098,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R657944a384d7485e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccd0d3277efd46ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6359,7 +6359,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc58a9876b813414e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8be0670716dc4023"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6935,7 +6935,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d5795a607634c13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3072f7ba233044a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7240,7 +7240,7 @@
         <x:v>Missing stays null</x:v>
       </x:c>
       <x:c r="F15" s="230" t="str">
-        <x:v>Validate response columnHeaders; never assume column order</x:v>
+        <x:v>Validate response columnHeaders; preserve signed integer Provider adjustments in RAW</x:v>
       </x:c>
       <x:c r="G15" s="231"/>
     </x:row>
@@ -7666,7 +7666,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58ad58b3b51d4b16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4d74200b87a4d1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7951,7 +7951,7 @@
         <x:v>Verify metric units</x:v>
       </x:c>
       <x:c r="C16" s="230" t="str">
-        <x:v>minutes×60, seconds direct, percentage÷100 evidence</x:v>
+        <x:v>signed integer adjustments preserved; minutes×60; seconds direct; percentage÷100 only in future canonical layer</x:v>
       </x:c>
       <x:c r="D16" s="230" t="str">
         <x:v>Blocking</x:v>
@@ -8246,7 +8246,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3989f69e169942b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f51aea5d7d450c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8522,7 +8522,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf9ce09d39f9410c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Readfaef2bd1546f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9807,7 +9807,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43be70b1b347406e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf510bd219fdc4a5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>